<commit_message>
Add Decap CMS: editable content layer (dates, guests, VIP, FAQ)
Content extracted from JSX into editable JSON (src/content/):
- event.json — forum dates, venue, gala time → wired into Hero (big date
  block, month/year, venue), TopBar, Footer
- special-guests.json → SpecialGuests.tsx
- vip.json (KZ + IT delegations) → VIP.tsx
- faq.json → FAQ.tsx

Decap CMS panel (public/admin/):
- index.html loads Decap 3 + Netlify Identity widget
- config.yml: git-gateway backend, ru locale, media→public/uploads,
  collections for event / special guests / VIP / FAQ with Russian field
  labels + hints for a non-dev editor

Netlify Identity widget added to root index.html (login → /admin redirect).

Build passes; admin/ ships in dist. Still TODO (needs Netlify UI, done by
user): link repo to Git, enable Identity + Git Gateway, invite editor.
Partners logos + remaining section texts to be added to CMS next.
</commit_message>
<xml_diff>
--- a/zayavki-investbridge.xlsx
+++ b/zayavki-investbridge.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Заявки" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Заявки'!$A$1:$K$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Заявки'!$A$1:$K$191</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K171"/>
+  <dimension ref="A1:K191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9233,8 +9233,1040 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>АО "Агентство "Хабар"</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>Оспанова Макпал Маулетовна</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>Менеджер по международным вопросам</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>Казахстан, г.Астана, ул.Кунаева,4</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>m.ospanova@khabar.kz</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>87172757624</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr"/>
+      <c r="K172" s="2" t="inlineStr">
+        <is>
+          <t>Информационный партнер</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>АО "РТРК Казахстан"</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>Алтынбек Рахметов</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>Продюсер ТВ</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>010000, Республика Казахстан, г. Астана, ул. Кунаева, д.4</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>press@rtrk.kz</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>+77768882323</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>https://rtrk.kz/en/</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr"/>
+      <c r="K173" s="2" t="inlineStr">
+        <is>
+          <t>государственная телерадиокорпорация, осуществляющая информационную политику нашего государства.
+Сегодня АО «РТРК «Казахстан» объединяет в своем составе: национальный телеканал «Qazaqstan», телеканалы «QAZSPORT», «Balapan», «Abai TV», «Казахское радио», радио «Шалқар», радио «Classic» (через ТОО «ҚАЗАҚ РАДИОЛАРЫ»), ТОО «Агенство Телевизионных Новостей» и региональные телерадиокомпании.
+Охват телеаудитории - 99 % населения страны, охват аудитории радиопередач - 88,74 % жителей Казахстана. Кроме того, сигналы АО «РТРК «Казахстан» могут принимать жители приграничных территорий сопредельных стран (Российская Федерация, Монгольская Народная Республика, Китайская Народная Республика, Кыргызская Республика, Республика Узбекистан).
+Эфирная сетка вещания телеканала «Qazaqstan» включает новости, сериалы, художественные, документальные фильмы и передачи. Медиаактивы АО «РТРК «Казахстан» удовлетворяют запросам широкой аудитории радиовещания и телевидения.
+Первый государственный спортивный телеканал «QAZSPORT» осуществляет прямые трансляции из всех регионов Казахстана, доступен в системе национального телевещания «Отау ТВ» и программах кабельных операторов. Спортивные трансляции на телеканале «QAZSPORT», включая трансляции чемпионатов Казахстана по ключевым и популярным видам спорта и прямые трансляции крупных зарубежных спортивных соревнований, составляют в размере 70% от общего объема вещания. Телеканал «QAZSPORT» вещает 20 часов в сутки.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>АО "Центр развития инвестиций" Qaragandy Invest "</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>Энергетика, транспорт, инфраструктура</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>Кудабаев Сунгат Болатович</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>И.О. Председателя правления</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>Казахстан. Кар.обл. Бухар-жырауский р-он, с.доскей , уч.квартал 028, здание 1662 блок 1</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>info@sez-saryarka.kz</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>+7 (701 ) 191 42 41</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>Q-invest.kz</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr"/>
+      <c r="K174" s="2" t="inlineStr">
+        <is>
+          <t>Компания занимается управлением проектов на территории СЭЗ где на сегодня работают более 20 предприятий в сфере производства промышленных товаров, химии, энергетики</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>QazTrade</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>Инвестиции, финансы, госорганы</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>Даурбаев Алиас Амангельдинович</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>Советник</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>ул. Достык 18, г. Астана</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>a.daurbayev@qaztrade.org.kz</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>+77770177721</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>qaztrade.org.kz</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>ДА</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="inlineStr">
+        <is>
+          <t>Внешняя торговля, привлечение экспортно-ориентированных инвестиций</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Kazakh Invest</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>Инвестиции, финансы, госорганы</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>Mekebayeva Anara</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>Acting Managing Director Task Force</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>Mangilik El str 55/20</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>a.mekebayeva@invest.gov.kz</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>87019994557</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>www.invest.gov.kz</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr"/>
+      <c r="K176" s="2" t="inlineStr">
+        <is>
+          <t>FDI attraction, realization of investment projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>КИ МИД</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>Инвестиции, финансы, госорганы</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>Мекебаева Сабина Артуровна</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>Стажер</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>Казахстан, Астана, Мангилик ел 55/1</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>sabinamekebayeva@icloud.com</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>8747943700</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr"/>
+      <c r="K177" s="2" t="inlineStr">
+        <is>
+          <t>attraction of FDI in KZ, realization of investment projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>ТОО SmartInvest LS</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>Инвестиции, финансы, госорганы</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>Tleubayev Arman</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>Astana</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>astanasell@mail.ru</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>87015274637</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr"/>
+      <c r="K178" s="2" t="inlineStr">
+        <is>
+          <t>Консалтинг в области ГЧП инвестиций</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>Внешнеторговая палата Казахстана</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>Даркембаев Алишер Ержанович</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>Директор департамента коммерческой деятельности</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>Казахстан, Астана, пр-т Туран 19/2</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>a.darkembayev@kazcic.kz</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>87018912261</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr"/>
+      <c r="K179" s="2" t="inlineStr">
+        <is>
+          <t>Внешнеторговая деятельность</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>ТОО AZ Syndicate</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>АПК и пищевая промышленность</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>Gulmira Kulpeissova</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>Regional Director</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Казахстан, г.Алматы, ул. Татибекова, 10</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>gkulpeissova@gmail.com</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>+77026120559</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/az_syndicate?igsh=eDJuZXQ1dHgzZHpl</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr"/>
+      <c r="K180" s="2" t="inlineStr">
+        <is>
+          <t>Прямой импорт из Италии и других европейский стран вина, б/а напитков и продуктов питания (гастрономия) в Казахстан. Дистрибьюция по Казахстану (HORECA и retail). Имеется собственная винотека Agora wine &amp; deli в Алмате.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>ICSC</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>Наука, образование, инновации</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>Lazzat Kussainova</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>Kazakhstan, Astana</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>ICSC2050@mail.ru</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>87716650372</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr"/>
+      <c r="K181" s="2" t="inlineStr">
+        <is>
+          <t>Популяризация науки, развитие научного образования</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>ТОО "Супермаркет " Солнечный "</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Арланов Владимир</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>Коммерческий директор</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>Казахстан, г.Костанай, ул.Карбышева, д.85</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>office@sunny.kz</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>87142932255</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>cc.kz</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr"/>
+      <c r="K182" s="2" t="inlineStr">
+        <is>
+          <t>Локальная сеть супермаркетов по продаже FMCG товаров г. Костанай</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>ALC Attorneys LLP</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>Айтбагин Фарит</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>Старший юрист</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>г. Астана, ул. Сыгана 60/2, БЦ Abu Dhabi Plaza</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>office@alc.legal</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>87023725856</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>alc.legal</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr"/>
+      <c r="K183" s="2" t="inlineStr">
+        <is>
+          <t>ALC Attorneys — международная юридическая фирма, работающая в Казахстане с 2011 года (офисы в Астане, Алматы, Актау, представительство в Баку) и в Узбекистане (Ташкент). Специализируемся на правовом сопровождении иностранных инвесторов: регистрация и структурирование компаний (включая AIFC/МФЦА), M&amp;A, лицензирование, энергетика и природные ресурсы, недвижимость, трудовое и миграционное право, а также судебное представительство при разрешении споров.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>ALC Attorneys LLP</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Алиев Фарид</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>Управляющий партнер</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>г. Астана, ул. Сыганак 60/2, БЦ Abu Dhabi Plaza</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>fa@alc.legal</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>87025056006</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>alc.legal</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr"/>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>ALC Attorneys — международная юридическая фирма, работающая в Казахстане с 2011 года (офисы в Астане, Алматы, Актау, представительство в Баку) и в Узбекистане (Ташкент). Специализируемся на правовом сопровождении иностранных инвесторов: регистрация и структурирование компаний (включая AIFC/МФЦА), M&amp;A, лицензирование, энергетика и природные ресурсы, недвижимость, трудовое и миграционное право, а также судебное представительство при разрешении споров.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>ALC Attroneys LLP</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>Жанадил Дана</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>Старший Партнер</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>г. Астана, ул. Сыганак 60/2, БЦ Abu Dhabi Plaza</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>dz@alc.legal</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>87010572483</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>alc.legal</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr"/>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>ALC Attorneys — международная юридическая фирма, работающая в Казахстане с 2011 года (офисы в Астане, Алматы, Актау, представительство в Баку) и в Узбекистане (Ташкент). Специализируемся на правовом сопровождении иностранных инвесторов: регистрация и структурирование компаний (включая AIFC/МФЦА), M&amp;A, лицензирование, энергетика и природные ресурсы, недвижимость, трудовое и миграционное право, а также судебное представительство при разрешении споров.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Maqsut Narikbayev University</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>Инвестиции, финансы, госорганы</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>Испенбетова Лилия Амангельдиевна</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>Government relations GR</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>Астана, Коргалжинское шоссе 8</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>ispenbetova@gmail.com</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>87053959720</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr"/>
+      <c r="K186" s="2" t="inlineStr">
+        <is>
+          <t>Университет
+Научные проекты 
+Проекты с ИИ 
+Мероприятия с гос.органами</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>IM.AG.IN. solutions srl</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Строительство, обрабатывающая промышленность</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>Хусаинова Алтын</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>Менеджер</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>Италия, Вия Рома 67, Медолаго (провинция Бергамо)</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>kaz@bonfanti.eu</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>+77028160333</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>www.bonfanti.eu</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr"/>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>Производство зерносушилок</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>Atlas Capital Management</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>Инвестиции, финансы, госорганы</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>Dinara Sheriyazdanova</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>Chief Investment Advisory</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>Сыганак 60/4</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>d.sheriyazdanova@atlascapital.kz</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>+77771454477</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr"/>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>Управляющая инвестиционная компания</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>TransAsia Logistic LLP</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>Энергетика, транспорт, инфраструктура</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>Майер Эвелина Андреевна</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>Переводчик</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>Астана, Казахстан</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>majerevelina7@gmail.com</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>+77767239708</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>https://translog.asia/</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr"/>
+      <c r="K189" s="2" t="inlineStr">
+        <is>
+          <t>Международный модальный экспортный оператор</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>AXAY Group</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>Бектурсын Хазретали</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>Директор</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Казахстан, Астана</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>khazretalib@bk.ru</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>+77773777650</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr"/>
+      <c r="K190" s="2" t="inlineStr">
+        <is>
+          <t>Международный трейдинг</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>Нефтегазовый совет Казахстана</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>Другое</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>Жолдыбаев Даниэль</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>Управляющий директор</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>Атырау, Сатпаева 45</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>d.zholdybayev@petrocouncil.kz</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>+77017443845</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>www.petrocouncil.kz</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr"/>
+      <c r="K191" s="2" t="inlineStr">
+        <is>
+          <t>Нефтегазовый Совет Казахстана «PetroCouncil» является одной из ведущих нефтегазовых ассоциации Казахстана.
+Petrocouncil.kz зарекомендовал себя одной из главной, надежной площадкой по развитию взаимодействия нефтегазовых операторов, компаний МСБ, а также государственных органов с целью развития местного содержания. Petrocouncil.kz тесно взаимодействует с нефтегазовыми компаниями, операторами, а также различными заинтересованными сторонами в регионе.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K171"/>
+  <autoFilter ref="A1:K191"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>